<commit_message>
Fix unstarted leagues to accurately report 0 completed matchdays and default Desde Jornada to 1
</commit_message>
<xml_diff>
--- a/data/Bundesliga.xlsx
+++ b/data/Bundesliga.xlsx
@@ -23,13 +23,27 @@
     <sheet sheetId="12" name="Jornada 32" state="visible" r:id="rId17"/>
     <sheet sheetId="13" name="Jornada 33" state="visible" r:id="rId18"/>
     <sheet sheetId="14" name="Jornada 34" state="visible" r:id="rId19"/>
+    <sheet sheetId="17" name="Jornada 1" state="visible" r:id="rId20"/>
+    <sheet sheetId="18" name="Jornada 2" state="visible" r:id="rId21"/>
+    <sheet sheetId="19" name="Jornada 3" state="visible" r:id="rId22"/>
+    <sheet sheetId="20" name="Jornada 4" state="visible" r:id="rId23"/>
+    <sheet sheetId="21" name="Jornada 5" state="visible" r:id="rId24"/>
+    <sheet sheetId="22" name="Jornada 6" state="visible" r:id="rId25"/>
+    <sheet sheetId="23" name="Jornada 7" state="visible" r:id="rId26"/>
+    <sheet sheetId="24" name="Jornada 8" state="visible" r:id="rId27"/>
+    <sheet sheetId="25" name="Jornada 9" state="visible" r:id="rId28"/>
+    <sheet sheetId="26" name="Jornada 10" state="visible" r:id="rId29"/>
+    <sheet sheetId="27" name="Jornada 11" state="visible" r:id="rId30"/>
+    <sheet sheetId="28" name="Jornada 12" state="visible" r:id="rId31"/>
+    <sheet sheetId="29" name="Jornada 13" state="visible" r:id="rId32"/>
+    <sheet sheetId="30" name="Jornada 14" state="visible" r:id="rId33"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2100" uniqueCount="133">
   <si>
     <t>Matchday</t>
   </si>
@@ -311,6 +325,123 @@
   </si>
   <si>
     <t>16/05/2026</t>
+  </si>
+  <si>
+    <t>Jornada 1</t>
+  </si>
+  <si>
+    <t>28/08/2026</t>
+  </si>
+  <si>
+    <t>29/08/2026</t>
+  </si>
+  <si>
+    <t>SC Paderborn</t>
+  </si>
+  <si>
+    <t>SV Elversberg</t>
+  </si>
+  <si>
+    <t>30/08/2026</t>
+  </si>
+  <si>
+    <t>FC Schalke 04</t>
+  </si>
+  <si>
+    <t>Jornada 2</t>
+  </si>
+  <si>
+    <t>04/09/2026</t>
+  </si>
+  <si>
+    <t>05/09/2026</t>
+  </si>
+  <si>
+    <t>06/09/2026</t>
+  </si>
+  <si>
+    <t>Jornada 3</t>
+  </si>
+  <si>
+    <t>11/09/2026</t>
+  </si>
+  <si>
+    <t>12/09/2026</t>
+  </si>
+  <si>
+    <t>13/09/2026</t>
+  </si>
+  <si>
+    <t>Jornada 4</t>
+  </si>
+  <si>
+    <t>18/09/2026</t>
+  </si>
+  <si>
+    <t>19/09/2026</t>
+  </si>
+  <si>
+    <t>20/09/2026</t>
+  </si>
+  <si>
+    <t>Jornada 5</t>
+  </si>
+  <si>
+    <t>10/10/2026</t>
+  </si>
+  <si>
+    <t>Jornada 6</t>
+  </si>
+  <si>
+    <t>17/10/2026</t>
+  </si>
+  <si>
+    <t>Jornada 7</t>
+  </si>
+  <si>
+    <t>24/10/2026</t>
+  </si>
+  <si>
+    <t>Jornada 8</t>
+  </si>
+  <si>
+    <t>31/10/2026</t>
+  </si>
+  <si>
+    <t>Jornada 9</t>
+  </si>
+  <si>
+    <t>07/11/2026</t>
+  </si>
+  <si>
+    <t>Jornada 10</t>
+  </si>
+  <si>
+    <t>21/11/2026</t>
+  </si>
+  <si>
+    <t>Jornada 11</t>
+  </si>
+  <si>
+    <t>28/11/2026</t>
+  </si>
+  <si>
+    <t>Jornada 12</t>
+  </si>
+  <si>
+    <t>05/12/2026</t>
+  </si>
+  <si>
+    <t>Jornada 13</t>
+  </si>
+  <si>
+    <t>12/12/2026</t>
+  </si>
+  <si>
+    <t>Jornada 14</t>
+  </si>
+  <si>
+    <t>19/12/2026</t>
   </si>
 </sst>
 </file>
@@ -2190,7 +2321,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2692,6 +2823,753 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>97</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>96</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>99</v>
+      </c>
+      <c r="D9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>99</v>
+      </c>
+      <c r="D10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s">
+        <v>100</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
+        <v>98</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>101</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" t="s">
+        <v>100</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" t="s">
+        <v>97</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F10" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G10"/>
@@ -2930,6 +3808,2496 @@
       </c>
       <c r="F10" t="s">
         <v>24</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" t="s">
+        <v>98</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F10" t="s">
+        <v>23</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>100</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>114</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>114</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>116</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>116</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>116</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>116</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" t="s">
+        <v>100</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>118</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>97</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>120</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>120</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>120</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
+        <v>100</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>121</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F10" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>97</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>124</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F10" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>126</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F10" t="s">
+        <v>100</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>127</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>128</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>128</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>127</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>128</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>130</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
+        <v>100</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>130</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F10" t="s">
+        <v>98</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -3187,6 +6555,255 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>131</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>132</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>131</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>132</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 

</xml_diff>